<commit_message>
EmailSetup updated test data and comments
</commit_message>
<xml_diff>
--- a/DataSource/TestData.xlsx
+++ b/DataSource/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\git\Travelbooking\travelbookingixigo\DataSource\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\Documents\APIAutomation\WebAndAPI\DataSource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80DEA8CD-AD71-437C-A493-0C10087FEE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08FBA1A-3AA3-4D92-B163-3E928A049009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TravellerInfo" sheetId="1" r:id="rId1"/>
@@ -613,10 +613,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="3">
-        <v>46230</v>
+        <v>46255</v>
       </c>
       <c r="E2" s="3">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="F2" t="s">
         <v>14</v>
@@ -701,10 +701,10 @@
         <v>16</v>
       </c>
       <c r="D4" s="3">
-        <v>46231</v>
+        <v>46262</v>
       </c>
       <c r="E4" s="3">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="F4" t="s">
         <v>33</v>
@@ -745,7 +745,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="20.6328125" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" customWidth="1"/>
+    <col min="3" max="3" width="16.7265625" customWidth="1"/>
     <col min="4" max="4" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -780,10 +780,10 @@
         <v>42</v>
       </c>
       <c r="C2" s="3">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="D2" s="3">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -803,10 +803,10 @@
         <v>43</v>
       </c>
       <c r="C3" s="3">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="D3" s="3">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -831,6 +831,7 @@
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
     <col min="2" max="2" width="10.36328125" customWidth="1"/>
     <col min="3" max="3" width="21.1796875" customWidth="1"/>
+    <col min="4" max="4" width="23.54296875" customWidth="1"/>
     <col min="5" max="5" width="15.08984375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -868,7 +869,7 @@
         <v>40</v>
       </c>
       <c r="C2" s="3">
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="D2" t="s">
         <v>52</v>
@@ -894,7 +895,7 @@
         <v>53</v>
       </c>
       <c r="C3" s="3">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="D3" t="s">
         <v>54</v>

</xml_diff>